<commit_message>
new cond files with new localizer design, main task (learn and retrieval) .psyexp added, new buffer concept (glasses) added
</commit_message>
<xml_diff>
--- a/psychopy_exp_files/sequences/retr_trials_prc_01.xlsx
+++ b/psychopy_exp_files/sequences/retr_trials_prc_01.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sync_folder\TSRlearn-LRI-online\sequences\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sync_folder\TSRlearn-MEG-prep\task\sequences\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
   <si>
     <t>trial_type</t>
   </si>
@@ -99,6 +99,12 @@
   </si>
   <si>
     <t>stimuli/practice_images/practice_sequence_overview_t1_03.jpg</t>
+  </si>
+  <si>
+    <t>iti_dur_retr</t>
+  </si>
+  <si>
+    <t>reflection_win_dur</t>
   </si>
 </sst>
 </file>
@@ -454,10 +460,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -494,8 +500,14 @@
       <c r="L1" t="s">
         <v>21</v>
       </c>
+      <c r="M1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N1" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -529,8 +541,14 @@
       <c r="L2" t="s">
         <v>22</v>
       </c>
+      <c r="M2">
+        <v>0.45</v>
+      </c>
+      <c r="N2">
+        <v>1.95</v>
+      </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -564,8 +582,14 @@
       <c r="L3" t="s">
         <v>23</v>
       </c>
+      <c r="M3">
+        <v>0.52</v>
+      </c>
+      <c r="N3">
+        <v>1.89</v>
+      </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
@@ -598,6 +622,12 @@
       </c>
       <c r="L4" t="s">
         <v>24</v>
+      </c>
+      <c r="M4">
+        <v>0.61</v>
+      </c>
+      <c r="N4">
+        <v>2.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>